<commit_message>
Download template with only the Sales_Data_Entry sheet.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/public/CyberSecurity_Sales_Template_With_Validation.xlsx
+++ b/public/CyberSecurity_Sales_Template_With_Validation.xlsx
@@ -1,26 +1,41 @@
 
-<file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
-  <workbookPr codeName="ThisWorkbook"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marin\Downloads\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55C3C7F5-636B-4A24-B766-D34175B50EFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
-  <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
-  </bookViews>
-  <sheets>
-    <sheet name="Sales_Data_Entry" sheetId="1" r:id="rId1"/>
-    <sheet name="Instructions" sheetId="2" r:id="rId2"/>
-  </sheets>
-  <calcPr calcId="0"/>
-</workbook>
+<file path=docProps\app.xml><?xml version="1.0" encoding="utf-8"?>
+<Properties xmlns="http://schemas.openxmlformats.org/officeDocument/2006/extended-properties" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
+  <Application>Microsoft Excel</Application>
+  <DocSecurity>0</DocSecurity>
+  <ScaleCrop>false</ScaleCrop>
+  <HeadingPairs>
+    <vt:vector size="2" baseType="variant">
+      <vt:variant>
+        <vt:lpstr>Worksheets</vt:lpstr>
+      </vt:variant>
+      <vt:variant>
+        <vt:i4>1</vt:i4>
+      </vt:variant>
+    </vt:vector>
+  </HeadingPairs>
+  <TitlesOfParts>
+    <vt:vector size="1" baseType="lpstr">
+      <vt:lpstr>Sales_Data_Entry</vt:lpstr>
+    </vt:vector>
+  </TitlesOfParts>
+  <LinksUpToDate>false</LinksUpToDate>
+  <SharedDoc>false</SharedDoc>
+  <HyperlinksChanged>false</HyperlinksChanged>
+  <AppVersion>16.0300</AppVersion>
+</Properties>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=docProps\core.xml><?xml version="1.0" encoding="utf-8"?>
+<cp:coreProperties xmlns:cp="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:dcmitype="http://purl.org/dc/dcmitype/" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
+  <dc:creator>openpyxl</dc:creator>
+  <cp:lastModifiedBy>Marina</cp:lastModifiedBy>
+  <dcterms:created xsi:type="dcterms:W3CDTF">2026-06-26T15:24:41Z</dcterms:created>
+  <dcterms:modified xsi:type="dcterms:W3CDTF">2026-09-29T12:47:29Z</dcterms:modified>
+</cp:coreProperties>
+</file>
+
+<file path=xl\sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="212" uniqueCount="145">
   <si>
     <t>Month</t>
@@ -460,7 +475,7 @@
 </sst>
 </file>
 
-<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
@@ -510,7 +525,7 @@
 </styleSheet>
 </file>
 
-<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\theme\theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
@@ -830,7 +845,27 @@
 </a:theme>
 </file>
 
-<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\workbook.xml><?xml version="1.0" encoding="utf-8"?>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <workbookPr codeName="ThisWorkbook"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marin\Downloads\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55C3C7F5-636B-4A24-B766-D34175B50EFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
+  <sheets>
+    <sheet name="Sales_Data_Entry" sheetId="1" r:id="rId1"/>
+  </sheets>
+  <calcPr calcId="0"/>
+</workbook>
+</file>
+
+<file path=xl\worksheets\sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AJ9"/>
   <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
@@ -1639,47 +1674,4 @@
     <ignoredError sqref="F1:J9 A1:D9 V1:AJ9 R1:R9" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:A6"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <sheetData>
-    <row r="1" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="3" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
-        <v>131</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <ignoredErrors>
-    <ignoredError sqref="A1:A6" numberStoredAsText="1"/>
-  </ignoredErrors>
-</worksheet>
 </file>
</xml_diff>